<commit_message>
La factura se guarda su propio detalle y la coleccion de Postman corre entera
El criterio del REQ-21 nombra siete entidades y solo habia seis: faltaba
detalle_facturas. Ahora la factura copia las lineas de la venta en el
momento de emitirla, asi que corregir manana el detalle de una venta ya no
reescribe lo que se facturo ayer. La migracion rellena las 97 lineas de las
facturas que ya existian.

El REQ-25 pide evidencia de Postman y la que habia era de pytest. La
coleccion queda en 86 peticiones con 97 comprobaciones y 0 fallos, y se
puede repetir: una carpeta de preparacion resuelve los identificadores
contra el catalogo vivo en lugar de traerlos escritos a mano, y el empleado
de prueba se crea con correo y documento distintos en cada corrida.

De paso, la casilla del ambiente estaba a medias y ahora dice 702.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evidencias/quinto_avance/Lista_Chequeo_Quinto_Avance_DILIGENCIADA.xlsx
+++ b/evidencias/quinto_avance/Lista_Chequeo_Quinto_Avance_DILIGENCIADA.xlsx
@@ -952,7 +952,7 @@
       <row>18</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5191125" cy="4143375"/>
+    <ext cx="5191125" cy="3762375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -1452,7 +1452,7 @@
       <row>38</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5191125" cy="3533775"/>
+    <ext cx="5191125" cy="4105275"/>
     <pic>
       <nvPicPr>
         <cNvPr id="26" name="Image 26" descr="Picture"/>
@@ -1919,7 +1919,7 @@
       <c r="E7" s="45" t="n"/>
       <c r="F7" s="34" t="inlineStr">
         <is>
-          <t xml:space="preserve">03 / Ambiente </t>
+          <t>03 / Ambiente 702</t>
         </is>
       </c>
       <c r="G7" s="45" t="n"/>
@@ -2115,11 +2115,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F15" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F15" s="19" t="n"/>
       <c r="G15" s="46" t="inlineStr">
         <is>
           <t>POST /api/ventas registra la venta con cliente, vendedor, productos, servicios, cantidades, descuentos, subtotal, IVA del 19%, total, forma de pago, fecha y estado. Los precios se leen del catalogo, nunca de la peticion. Descuenta inventario y anular lo devuelve. Se puede registrar desde el panel o desde el carrito del sitio.</t>
@@ -2152,11 +2148,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F16" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F16" s="19" t="n"/>
       <c r="G16" s="47" t="inlineStr">
         <is>
           <t>Tabla detalle_ventas: una fila por articulo con tipo (producto o servicio), cantidad, precio unitario, descuento y subtotal. Guarda copia del nombre y del precio del momento, asi el historico no cambia si el articulo se edita o se retira del catalogo.</t>
@@ -2189,11 +2181,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F17" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F17" s="19" t="n"/>
       <c r="G17" s="46" t="inlineStr">
         <is>
           <t>GET /api/ventas filtra por fecha inicial y final, cliente, producto, servicio, estado, forma de pago, valor minimo y maximo, y texto libre sobre numero de venta, nombre, correo o documento. El cliente solo recibe sus propias compras.</t>
@@ -2226,18 +2214,14 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F18" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F18" s="19" t="n"/>
       <c r="G18" s="47" t="inlineStr">
         <is>
           <t>GET /api/reportes/ventas-diarias devuelve fecha, numero de venta, cliente, productos y servicios, cantidad, valor, total y estado. Los tres formatos (pantalla, PDF y Excel) salen de un unico calculo, para que no puedan discrepar entre si.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="330.6" customHeight="1" s="43">
+    <row r="19" ht="300.2" customHeight="1" s="43">
       <c r="A19" s="24" t="inlineStr">
         <is>
           <t>REQ-05</t>
@@ -2263,11 +2247,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F19" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F19" s="19" t="n"/>
       <c r="G19" s="46" t="inlineStr">
         <is>
           <t>Generado con ReportLab. Incluye nombre y NIT del negocio, fecha del reporte, tabla de ventas, totales con IVA y sello de generacion. Se pagina solo si el dia tiene muchas ventas. Las anuladas aparecen listadas pero no suman al total.</t>
@@ -2300,11 +2280,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F20" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F20" s="19" t="n"/>
       <c r="G20" s="47" t="inlineStr">
         <is>
           <t>Generado con openpyxl. Tres hojas: Ventas, Detalle (una fila por articulo, para analizar) y Resumen. Trae autofiltro, primera fila congelada, formato de moneda y formulas =SUM() vivas, de modo que al filtrar los totales se recalculan solos.</t>
@@ -2337,11 +2313,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F21" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F21" s="19" t="n"/>
       <c r="G21" s="46" t="inlineStr">
         <is>
           <t>La factura nace de una venta registrada y lleva numero consecutivo (FV-2026-000061), fecha, datos del cliente, detalle con cantidad y precio unitario, subtotal, IVA y total. Copia los datos del cliente al emitirse: es un documento y no cambia despues.</t>
@@ -2374,11 +2346,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F22" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F22" s="19" t="n"/>
       <c r="G22" s="47" t="inlineStr">
         <is>
           <t>GET /api/facturas busca por numero de factura, nombre, documento o correo del cliente, rango de fechas y estado. El cliente ve unicamente las suyas, y el recorte lo hace FastAPI a partir del rol del token.</t>
@@ -2411,11 +2379,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F23" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F23" s="19" t="n"/>
       <c r="G23" s="46" t="inlineStr">
         <is>
           <t>GET /api/facturas/{id}/pdf entrega el documento con Content-Disposition. Se descarga desde el panel del administrador, desde el del empleado y desde el del propio cliente, que solo puede bajar las suyas.</t>
@@ -2448,11 +2412,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F24" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F24" s="19" t="n"/>
       <c r="G24" s="47" t="inlineStr">
         <is>
           <t>Tarjetas tipo Card con usuarios, catalogo, ventas del periodo, facturacion, ventas de hoy, acumulado del mes, valor del inventario y PQR recibidas con las que siguen sin cerrar.</t>
@@ -2485,11 +2445,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F25" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F25" s="19" t="n"/>
       <c r="G25" s="46" t="inlineStr">
         <is>
           <t>Grafico de barras y grafico lineal sobre la misma serie, mas los Cards de indicadores y los repartos por estado y forma de pago. Se puede agrupar por dia, semana o mes. Estan dibujados en SVG propio, sin sumar ninguna libreria al proyecto.</t>
@@ -2522,11 +2478,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F26" s="19" t="n"/>
       <c r="G26" s="47" t="inlineStr">
         <is>
           <t>Administrador, Empleado y Cliente llaman al mismo endpoint y reciben respuestas distintas. El empleado no ve el conteo de usuarios y el cliente solo ve sus propias cifras: el inventario y los totales del negocio le llegan en null.</t>
@@ -2559,11 +2511,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F27" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F27" s="19" t="n"/>
       <c r="G27" s="46" t="inlineStr">
         <is>
           <t>Fecha inicial y final, agrupacion, estado, forma de pago, articulo y cliente. En la captura estan aplicados agrupacion por semana y estado Pagadas: el indicador baja de 60 a 50 ventas y el grafico pasa a barras semanales.</t>
@@ -2596,11 +2544,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F28" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F28" s="19" t="n"/>
       <c r="G28" s="47" t="inlineStr">
         <is>
           <t>21 endpoints nuevos (45 en total) repartidos en ventas, facturas, reportes, PQR, estadisticas y chatbot, documentados en Swagger con sus codigos de respuesta.</t>
@@ -2633,11 +2577,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F29" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F29" s="19" t="n"/>
       <c r="G29" s="46" t="inlineStr">
         <is>
           <t>Ninguna cifra esta escrita a mano en React: todo viene de GET /api/estadisticas/resumen y /api/estadisticas/ventas. La captura muestra los tres tokens contra el mismo endpoint y las respuestas distintas que devuelve.</t>
@@ -2670,11 +2610,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F30" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F30" s="19" t="n"/>
       <c r="G30" s="47" t="inlineStr">
         <is>
           <t>El cliente radica peticion, queja, reclamo o sugerencia y recibe un numero de radicado (PQR-2026-000001). Cuatro estados: pendiente, en proceso, respondida y cerrada. El equipo responde y queda registrado quien atendio y cuando.</t>
@@ -2707,11 +2643,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F31" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F31" s="19" t="n"/>
       <c r="G31" s="46" t="inlineStr">
         <is>
           <t>Chatbot flotante en todo el sitio publico. Atiende tambien a visitantes sin cuenta, responde con el catalogo real de la base de datos, orienta el proceso de compra y encauza las PQR. Las conversaciones quedan guardadas en las tablas conversaciones y mensajes.</t>
@@ -2744,11 +2676,7 @@
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="F32" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F32" s="19" t="n"/>
       <c r="G32" s="47" t="inlineStr">
         <is>
           <t>La integracion esta construida y probada: FastAPI llama al proveedor (Anthropic u OpenAI, y cualquier API compatible cambiando IA_URL_BASE), le entrega el catalogo real como contexto y guarda el modelo que respondio en cada mensaje. Hay pruebas automaticas con el proveedor simulado. FALTA unicamente cargar una API Key en IA_API_KEY: sin ella el chatbot responde con su motor de reglas, que consulta la misma base de datos.</t>
@@ -2781,11 +2709,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F33" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F33" s="19" t="n"/>
       <c r="G33" s="46" t="inlineStr">
         <is>
           <t>IA_API_KEY se lee de variables de entorno mediante pydantic-settings. El archivo .env esta en .gitignore y no hay ninguno versionado: en el repositorio solo viajan los .env.example sin valores. GET /api/chatbot/estado informa si hay clave configurada pero nunca la devuelve, y los errores del proveedor se registran sin el cuerpo de la peticion.</t>
@@ -2818,11 +2742,7 @@
           <t>En Proceso</t>
         </is>
       </c>
-      <c r="F34" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F34" s="19" t="n"/>
       <c r="G34" s="47" t="inlineStr">
         <is>
           <t>La configuracion esta lista y ensayada en local: railway.json y Procfile de cada servicio, Dockerfile como alternativa, servidor.js que resuelve las rutas de React Router en produccion, DATABASE_URL de la plataforma convertida al driver de SQLAlchemy y CORS por variable de entorno. Se probo el Frontend compilado contra el Backend en ENTORNO=produccion: enlaces directos sin 404 y preflight CORS correcto. FALTA ejecutar el despliegue y publicar la URL, que requiere crear las cuentas. Paso a paso en DESPLIEGUE.md.</t>
@@ -2855,14 +2775,10 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F35" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F35" s="19" t="n"/>
       <c r="G35" s="46" t="inlineStr">
         <is>
-          <t>La base pasa de 7 a 13 tablas. Se agregan ventas, detalle_ventas, facturas, pqr, conversaciones y mensajes, con sus claves foraneas declaradas en la propia base. database/quinto_avance.sql es aditivo, para no perder los datos de los avances anteriores.</t>
+          <t>La base pasa de 7 a 14 tablas. Se agregan las siete entidades del criterio: ventas, detalle_ventas, facturas, detalle_facturas, pqr, conversaciones y mensajes, con sus claves foraneas declaradas en la propia base, no solo en el ORM. detalle_facturas guarda copia de las lineas al emitir: junto con los datos del cliente y los totales que ya copiaba la factura, el documento deja de depender de la venta. database/quinto_avance.sql es aditivo, para no perder los datos de avances anteriores.</t>
         </is>
       </c>
     </row>
@@ -2892,11 +2808,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F36" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F36" s="19" t="n"/>
       <c r="G36" s="47" t="inlineStr">
         <is>
           <t>Se mantiene la separacion entre modelos ORM (SQLAlchemy, describen la tabla) y esquemas Pydantic (validan lo que entra y dan forma a lo que sale). Cinco modelos nuevos y seis archivos de esquemas para ventas, facturas, PQR, chat, reportes y estadisticas.</t>
@@ -2929,11 +2841,7 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F37" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F37" s="19" t="n"/>
       <c r="G37" s="46" t="inlineStr">
         <is>
           <t>Los tres paneles se arman con los mismos componentes: MarcoPanel, Dashboard, TablaVentas, TablaFacturas, PanelPqr, PanelReportes, los graficos y las tarjetas. Cambia la lista de secciones que recibe cada rol, no el codigo. Todo conserva el sistema de diseno de los avances anteriores.</t>
@@ -2966,18 +2874,14 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F38" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F38" s="19" t="n"/>
       <c r="G38" s="47" t="inlineStr">
         <is>
           <t>El mismo endpoint responde 401 sin token, 403 con token de rol insuficiente o invalido, y 200 con el correcto. Contrasenas con hash bcrypt de 12 rondas, credenciales en variables de entorno y topes en los endpoints publicos: 3 enlaces de recuperacion por correo cada 15 minutos y 25 mensajes de chatbot por equipo cada 10 minutos.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="281.96" customHeight="1" s="43">
+    <row r="39" ht="327.56" customHeight="1" s="43">
       <c r="A39" s="24" t="inlineStr">
         <is>
           <t>REQ-25</t>
@@ -3003,14 +2907,10 @@
           <t>Cumplido</t>
         </is>
       </c>
-      <c r="F39" s="19" t="inlineStr">
-        <is>
-          <t>[Pegar Captura de Pantalla Aquí]</t>
-        </is>
-      </c>
+      <c r="F39" s="19" t="n"/>
       <c r="G39" s="46" t="inlineStr">
         <is>
-          <t>Coleccion de Postman con 84 peticiones en 12 carpetas (backend/postman/). Ademas, scripts/verificar_quinto_avance.py recorre la API contra MySQL real comprobando tanto lo que debe funcionar como lo que debe ser rechazado, y deja anuladas las ventas que crea. Se suman 130 pruebas automaticas con pytest.</t>
+          <t>Coleccion de Postman con 86 peticiones en 13 carpetas, ejecutada con newman (la CLI oficial de Postman): 97 aserciones, 0 fallos. Ejercita los cinco metodos: GET 45, POST 26, PATCH 8, DELETE 4 y PUT 3. La coleccion resuelve sola los identificadores contra el catalogo y genera datos unicos en cada ejecucion, asi que se puede repetir sin chocar consigo misma. Se suman 133 pruebas automaticas con pytest y el recorrido de scripts/verificar_quinto_avance.py contra MySQL real.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
El chatbot ya responde con Inteligencia Artificial (REQ-18)
Queda conectado a Groq, que expone una API compatible con la de OpenAI, asi
que basto con apuntar IA_URL_BASE: no hizo falta tocar el codigo. El modelo
es openai/gpt-oss-120b.

La evidencia se rehizo con datos tomados en vivo, porque la anterior
mostraba ia_activa en false. Ahora se ve la llamada al proveedor, el estado
del endpoint y una conversacion real en la que el modelo cita precios y
unidades que salen de la base MySQL, no de su imaginacion.

La lista de chequeo pasa de 23 a 24 cumplidos (96%). El unico que sigue en
proceso es el despliegue, que espera una URL publica.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evidencias/quinto_avance/Lista_Chequeo_Quinto_Avance_DILIGENCIADA.xlsx
+++ b/evidencias/quinto_avance/Lista_Chequeo_Quinto_Avance_DILIGENCIADA.xlsx
@@ -1277,7 +1277,7 @@
       <row>31</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5191125" cy="3829050"/>
+    <ext cx="5191125" cy="5286375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="19" name="Image 19" descr="Picture"/>
@@ -2650,7 +2650,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="305.52" customHeight="1" s="43">
+    <row r="32" ht="421.8" customHeight="1" s="43">
       <c r="A32" s="25" t="inlineStr">
         <is>
           <t>REQ-18</t>
@@ -2673,13 +2673,13 @@
       </c>
       <c r="E32" s="18" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="F32" s="19" t="n"/>
       <c r="G32" s="47" t="inlineStr">
         <is>
-          <t>La integracion esta construida y probada: FastAPI llama al proveedor (Anthropic u OpenAI, y cualquier API compatible cambiando IA_URL_BASE), le entrega el catalogo real como contexto y guarda el modelo que respondio en cada mensaje. Hay pruebas automaticas con el proveedor simulado. FALTA unicamente cargar una API Key en IA_API_KEY: sin ella el chatbot responde con su motor de reglas, que consulta la misma base de datos.</t>
+          <t>El chatbot responde con Inteligencia Artificial: FastAPI llama al proveedor desde el servidor, le entrega el catalogo real como contexto y guarda en cada mensaje el modelo que respondio. Funcionando con openai/gpt-oss-120b a traves de Groq, que expone una API compatible con la de OpenAI; basta cambiar IA_URL_BASE para usar Anthropic, OpenAI u otro proveedor. La captura muestra una conversacion real donde el modelo cita precios y unidades tomados de la base MySQL, no inventados. Si falta la clave el chatbot no se cae: vuelve solo a su motor de reglas, que consulta esa misma base.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
La aplicacion queda desplegada y en funcionamiento (REQ-20)
Frontend en Vercel, Backend en Render y MySQL en Aiven: tres proveedores
distintos hablando por HTTPS. Con esto la lista de chequeo llega a 25 de 25.

No se da por bueno el despliegue solo porque las paginas carguen. Se verifico
contra los dominios publicos: /salud responde con la base conectada, el
entorno ya es produccion, el catalogo sirve las 12 motocicletas, el login
entrega token, los Dashboards traen indicadores, los reportes bajan en PDF y
en Excel, el chatbot responde con IA citando precios reales, y el preflight
CORS autoriza el dominio del Frontend -que era justo lo que faltaba y tenia
el catalogo en blanco-.

La evidencia se rehizo con capturas tomadas del sitio ya publicado.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evidencias/quinto_avance/Lista_Chequeo_Quinto_Avance_DILIGENCIADA.xlsx
+++ b/evidencias/quinto_avance/Lista_Chequeo_Quinto_Avance_DILIGENCIADA.xlsx
@@ -1327,7 +1327,7 @@
       <row>33</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5191125" cy="3248025"/>
+    <ext cx="5191125" cy="5715000"/>
     <pic>
       <nvPicPr>
         <cNvPr id="21" name="Image 21" descr="Picture"/>
@@ -2716,7 +2716,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="259.16" customHeight="1" s="43">
+    <row r="34" ht="456" customHeight="1" s="43">
       <c r="A34" s="25" t="inlineStr">
         <is>
           <t>REQ-20</t>
@@ -2739,13 +2739,13 @@
       </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="F34" s="19" t="n"/>
       <c r="G34" s="47" t="inlineStr">
         <is>
-          <t>La configuracion esta lista y ensayada en local: railway.json y Procfile de cada servicio, Dockerfile como alternativa, servidor.js que resuelve las rutas de React Router en produccion, DATABASE_URL de la plataforma convertida al driver de SQLAlchemy y CORS por variable de entorno. Se probo el Frontend compilado contra el Backend en ENTORNO=produccion: enlaces directos sin 404 y preflight CORS correcto. FALTA ejecutar el despliegue y publicar la URL, que requiere crear las cuentas. Paso a paso en DESPLIEGUE.md.</t>
+          <t>Aplicacion desplegada y en funcionamiento. Frontend en Vercel: https://motoshub-react-fastapi.vercel.app ; Backend en Render: https://motoshub-react-fastapi.onrender.com ; base de datos MySQL en Aiven, con las 14 tablas y el historial de demostracion. Verificado en produccion: /salud responde "base_datos": "conectada", el entorno es "produccion", el catalogo sirve las 12 motocicletas, el login entrega token, los Dashboards traen indicadores, los reportes bajan en PDF y en Excel, el chatbot responde con IA y el preflight CORS autoriza el dominio del Frontend. Paso a paso reproducible en DESPLIEGUE.md.</t>
         </is>
       </c>
     </row>

</xml_diff>